<commit_message>
test(module1): 精简冗余用例 015/023/041（43→40 条）
背景与目标：对全部用例做冗余分析，删掉三条不产生独有覆盖的用例。
实测（临时副本逐条删除后测量）：删除后被测源码覆盖率完全不变
（804 语句/382 分支、54%，TOTAL 57%），通过数 40。

主要改动：
- testdata/cron_cases.json：删除 CRON-UT-015（与 021 同表达式同预期，
  021 起点恰在触发点上、语义更强）、CRON-UT-023（正午 12 点非边界值，
  边界值方法归类不成立）、CRON-UT-041（与 011 同属字段越界等价类）
- testcases/附录1-测试用例清单v3.xlsx：删除对应三行，概述与修订记录 3.04
- 同步 requirements_traceability.md、module1/README.md、tests/testdata/
  testcases 的 README、专项检查转换用例说明.md（041 条目标注删除原因）、
  docs/项目结构说明.md：43→40 条用例、40 passed

验证：修复后源码 40 passed、branch coverage 57%（与精简前一致）；
基线源码 3 failed（033/034/035）、37 passed，缺陷检测不受影响。
清单 v3 经 openpyxl 重载校验 40 行，图片与统计公式保留。

待办：presentation/output/模块一成果汇报v2.pptx 因被 PowerPoint 占用
暂未同步（仍为 43 条口径），待文件关闭后更新。
</commit_message>
<xml_diff>
--- a/module1/testcases/附录1-测试用例清单v3.xlsx
+++ b/module1/testcases/附录1-测试用例清单v3.xlsx
@@ -1889,7 +1889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L46"/>
+  <dimension ref="A2:L47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.6296296296296" defaultRowHeight="15.75"/>
   <cols>
     <col width="1.62962962962963" customWidth="1" style="9" min="1" max="1"/>
@@ -2104,7 +2104,7 @@
       <c r="D15" s="17" t="n"/>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>对 croniter 的表达式解析、迭代、匹配、范围与时区执行 43 个清单参数化用例(CRON-UT-001—011、013—025、033—035、037—052,原 5 条专项自动化检查已并入账本);用例按设计方法归类为等价类、边界值与场景法三类,其中夏令时覆盖切换日、跳变时刻与回拨歧义小时,并与《手动测试v2.md》《自动化测试设计与实施说明v2.md》及 testdata/cron_cases.json 同步。</t>
+          <t>对 croniter 的表达式解析、迭代、匹配、范围与时区执行 40 个清单参数化用例(原 5 条专项自动化检查已并入账本;已删除冗余用例 012、015、023、026—032、036、041);用例按设计方法归类为等价类、边界值与场景法三类,其中夏令时覆盖切换日、跳变时刻与回拨歧义小时,并与《手动测试v2.md》《自动化测试设计与实施说明v2.md》及 testdata/cron_cases.json 同步。</t>
         </is>
       </c>
       <c r="F15" s="17" t="n"/>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>3.04</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>v3.03:新增 CRON-UT-051/052 两条夏令时边界用例(春季跳变日跳过不存在的 02:00、秋季回拨日歧义小时取第一次);043 以切换前一天为基准仅验证普通时区触发,跳变行为由 051/052 补齐;总数 41→43</t>
+          <t>v3.04:精简冗余用例——015(与 021 同表达式同预期,被严格覆盖)、023(12 点非边界值,方法归类不成立)、041(与 011 同属字段越界等价类);删除后 40 条,通过 40/40,分支覆盖率不变</t>
         </is>
       </c>
       <c r="K26" s="19" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C27" s="28" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2417,12 +2417,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="21" t="n"/>
-      <c r="G27" s="21" t="n"/>
-      <c r="H27" s="21" t="n"/>
-      <c r="I27" s="21" t="n"/>
-      <c r="J27" s="21" t="n"/>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>v3.03:新增 CRON-UT-051/052 两条夏令时边界用例(春季跳变日跳过不存在的 02:00、秋季回拨日歧义小时取第一次);043 以切换前一天为基准仅验证普通时区触发,跳变行为由 051/052 补齐;总数 41→43</t>
+        </is>
+      </c>
       <c r="K27" s="19" t="inlineStr">
         <is>
           <t>测试小组</t>
@@ -2437,7 +2436,7 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -2445,11 +2444,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>v3.01:将 5 条专项自动化检查并入账本参数化(新增 CRON-UT-041—050:日期越界、秒级返回类型、夏令时、非法输入类型、match/match_range/croniter_range/is_valid);删除 5 个独立测试函数;总数 41 清单用例=41 pytest 用例</t>
-        </is>
-      </c>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="21" t="n"/>
+      <c r="I28" s="21" t="n"/>
+      <c r="J28" s="21" t="n"/>
       <c r="K28" s="19" t="inlineStr">
         <is>
           <t>测试小组</t>
@@ -2464,97 +2464,101 @@
       </c>
       <c r="C29" s="28" t="inlineStr">
         <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>v3.01:将 5 条专项自动化检查并入账本参数化(新增 CRON-UT-041—050:日期越界、秒级返回类型、夏令时、非法输入类型、match/match_range/croniter_range/is_valid);删除 5 个独立测试函数;总数 41 清单用例=41 pytest 用例</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>测试小组</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="54" t="inlineStr">
+        <is>
+          <t>2026.09.10</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
           <t>3.02</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>v3.02:045—050 的类别由接口名 match 修正为设计方法(045—049→等价类、050→场景法),检查类型改由 check 字段承载;备注列同步改为方法名</t>
         </is>
       </c>
-      <c r="K29" s="19" t="inlineStr">
+      <c r="K30" s="19" t="inlineStr">
         <is>
           <t>测试小组</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="17" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Distribution LIST 分发记录</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-      <c r="K30" s="17" t="n"/>
-      <c r="L30" s="18" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t>Copy No.</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>Holder's Name &amp; Role  持有者和角色</t>
-        </is>
-      </c>
+      <c r="C31" s="17" t="n"/>
       <c r="D31" s="17" t="n"/>
       <c r="E31" s="17" t="n"/>
       <c r="F31" s="17" t="n"/>
       <c r="G31" s="17" t="n"/>
       <c r="H31" s="17" t="n"/>
       <c r="I31" s="17" t="n"/>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>Issue Date  分发日期</t>
-        </is>
-      </c>
+      <c r="J31" s="17" t="n"/>
       <c r="K31" s="17" t="n"/>
       <c r="L31" s="18" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>&lt;T.M.B&amp;C.P.M&gt;</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="19" t="n"/>
-      <c r="F32" s="19" t="n"/>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="19" t="n"/>
-      <c r="J32" s="54" t="inlineStr">
-        <is>
-          <t>yyyy.mm.dd</t>
-        </is>
-      </c>
-      <c r="K32" s="54" t="n"/>
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>Copy No.</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Holder's Name &amp; Role  持有者和角色</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>Issue Date  分发日期</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="n"/>
       <c r="L32" s="18" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>&lt;Project Manager&gt;</t>
+          <t>&lt;T.M.B&amp;C.P.M&gt;</t>
         </is>
       </c>
       <c r="D33" s="19" t="n"/>
@@ -2573,11 +2577,11 @@
     </row>
     <row r="34">
       <c r="B34" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>&lt;Team members&gt;</t>
+          <t>&lt;Project Manager&gt;</t>
         </is>
       </c>
       <c r="D34" s="19" t="n"/>
@@ -2596,11 +2600,11 @@
     </row>
     <row r="35">
       <c r="B35" s="19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>&lt;Customer Representative&gt;</t>
+          <t>&lt;Team members&gt;</t>
         </is>
       </c>
       <c r="D35" s="19" t="n"/>
@@ -2618,142 +2622,155 @@
       <c r="L35" s="18" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="31" t="n">
+      <c r="B36" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>&lt;Customer Representative&gt;</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="54" t="inlineStr">
+        <is>
+          <t>yyyy.mm.dd</t>
+        </is>
+      </c>
+      <c r="K36" s="54" t="n"/>
+      <c r="L36" s="18" t="n"/>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="B37" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C37" s="32" t="inlineStr">
         <is>
           <t>&lt;Others&gt;</t>
         </is>
       </c>
-      <c r="D36" s="32" t="n"/>
-      <c r="E36" s="32" t="n"/>
-      <c r="F36" s="32" t="n"/>
-      <c r="G36" s="32" t="n"/>
-      <c r="H36" s="32" t="n"/>
-      <c r="I36" s="32" t="n"/>
-      <c r="J36" s="56" t="inlineStr">
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="56" t="inlineStr">
         <is>
           <t>yyyy.mm.dd</t>
         </is>
       </c>
-      <c r="K36" s="57" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="B37" s="35" t="n"/>
-      <c r="C37" s="35" t="n"/>
-      <c r="D37" s="35" t="n"/>
-      <c r="E37" s="35" t="n"/>
-      <c r="F37" s="35" t="n"/>
-      <c r="G37" s="35" t="n"/>
-      <c r="H37" s="35" t="n"/>
-      <c r="I37" s="35" t="n"/>
-      <c r="J37" s="58" t="n"/>
-      <c r="K37" s="58" t="n"/>
-    </row>
-    <row r="38"/>
+      <c r="K37" s="57" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="35" t="n"/>
+      <c r="F38" s="35" t="n"/>
+      <c r="G38" s="35" t="n"/>
+      <c r="H38" s="35" t="n"/>
+      <c r="I38" s="35" t="n"/>
+      <c r="J38" s="58" t="n"/>
+      <c r="K38" s="58" t="n"/>
+    </row>
     <row r="39"/>
-    <row r="40">
-      <c r="B40" s="37" t="inlineStr">
+    <row r="40"/>
+    <row r="41">
+      <c r="B41" s="37" t="inlineStr">
         <is>
           <t>测试结果分析</t>
         </is>
       </c>
-      <c r="C40" s="38" t="n"/>
-      <c r="D40" s="38" t="n"/>
-      <c r="E40" s="39" t="n"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="40" t="inlineStr">
+      <c r="C41" s="38" t="n"/>
+      <c r="D41" s="38" t="n"/>
+      <c r="E41" s="39" t="n"/>
+    </row>
+    <row r="42" ht="3" customHeight="1">
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>OK项</t>
         </is>
       </c>
-      <c r="C41" s="41">
+      <c r="C42" s="41">
         <f>IF($E$13=0,0,COUNTIF('Test Cases测试用例'!$L:$L,"=OK"))</f>
         <v/>
       </c>
-      <c r="D41" s="40" t="inlineStr">
+      <c r="D42" s="40" t="inlineStr">
         <is>
           <t>OK率</t>
         </is>
       </c>
-      <c r="E41" s="42">
+      <c r="E42" s="42">
         <f>IF(E13=0,0,C38/E13)</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="3" customHeight="1">
-      <c r="B42" s="40" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="40" t="inlineStr">
         <is>
           <t>POK项</t>
         </is>
       </c>
-      <c r="C42" s="41">
+      <c r="C43" s="41">
         <f>IF($E$13=0,0,COUNTIF('Test Cases测试用例'!$L:$L,"=POK"))</f>
         <v/>
       </c>
-      <c r="D42" s="40" t="inlineStr">
+      <c r="D43" s="40" t="inlineStr">
         <is>
           <t>POK率</t>
         </is>
       </c>
-      <c r="E42" s="42">
+      <c r="E43" s="42">
         <f>IF(E13=0,0,C39/E13)</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="40" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="40" t="inlineStr">
         <is>
           <t>NG项</t>
         </is>
       </c>
-      <c r="C43" s="41">
+      <c r="C44" s="41">
         <f>IF($E$13=0,0,COUNTIF('Test Cases测试用例'!$L:$L,"=NG"))</f>
         <v/>
       </c>
-      <c r="D43" s="40" t="inlineStr">
-        <is>
-          <t>NG率</t>
-        </is>
-      </c>
-      <c r="E43" s="42">
-        <f>IF(E13=0,0,C40/E13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="43" t="inlineStr">
+      <c r="D44" s="38" t="n"/>
+      <c r="E44" s="39" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="43" t="inlineStr">
         <is>
           <t>NT项</t>
         </is>
       </c>
-      <c r="C44" s="44">
+      <c r="C45" s="44">
         <f>IF($E$13=0,0,COUNTIF('Test Cases测试用例'!$L:$L,"=NT"))</f>
         <v/>
       </c>
-      <c r="D44" s="60" t="n"/>
-      <c r="E44" s="61" t="n"/>
-    </row>
-    <row r="45">
-      <c r="B45" s="46" t="n"/>
-      <c r="C45" s="59" t="n"/>
-      <c r="D45" s="38" t="n"/>
-      <c r="E45" s="39" t="n"/>
+      <c r="D45" s="60" t="n"/>
+      <c r="E45" s="61" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="50" t="inlineStr">
+      <c r="B46" s="46" t="n"/>
+      <c r="C46" s="59" t="n"/>
+      <c r="D46" s="38" t="n"/>
+      <c r="E46" s="39" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="50" t="inlineStr">
         <is>
           <t>用例总个数</t>
         </is>
       </c>
-      <c r="C46" s="51">
+      <c r="C47" s="51">
         <f>E13</f>
         <v/>
       </c>
-      <c r="D46" s="52" t="n"/>
-      <c r="E46" s="53" t="n"/>
+      <c r="D47" s="52" t="n"/>
+      <c r="E47" s="53" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2771,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.6296296296296" defaultRowHeight="15.75"/>
   <cols>
     <col width="15.362962962963" customWidth="1" style="8" min="1" max="1"/>
@@ -3614,22 +3631,22 @@
     <row r="13" ht="150" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-041</t>
+          <t>CRON-UT-013</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>croniter() 解析</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>等价类:日期越界 0 0 32 * * 应抛出标准错误</t>
+          <t>get_next()/get_prev() 迭代</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>边界值:每分钟迭代(起始 00:00,分钟边界)</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -3649,26 +3666,22 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 32 * *(日 32 越界);start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=* * * * *;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>try:
-    croniter('0 0 32 * *', start)
-    print('未抛异常，该用例失败')
-except CroniterBadCronError as e:
-    print('CroniterBadCronError:', e)</t>
+          <t>croniter('* * * * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>CroniterBadCronError: [0 0 32 * *] is not acceptable, out of range</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 1, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
-          <t>CroniterBadCronError: [0 0 32 * *] is not acceptable, out of range</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 1, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L13" s="12" t="inlineStr">
@@ -3678,14 +3691,14 @@
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>等价类(非法表达式类,日期越界)</t>
+          <t>边界值(分钟边界)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="75" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-013</t>
+          <t>CRON-UT-014</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -3695,7 +3708,7 @@
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>边界值:每分钟迭代(起始 00:00,分钟边界)</t>
+          <t>边界值:整点迭代(起始 00:00,小时边界)</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -3720,22 +3733,22 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>expr=* * * * *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 * * * *;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>croniter('* * * * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 * * * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 1, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 1, 1, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 1, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 1, 1, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L14" s="12" t="inlineStr">
@@ -3745,14 +3758,14 @@
       </c>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>边界值(分钟边界)</t>
+          <t>边界值(小时边界)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="75" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-014</t>
+          <t>CRON-UT-016</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -3762,7 +3775,7 @@
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>边界值:整点迭代(起始 00:00,小时边界)</t>
+          <t>边界值:闰年 2 月 29 日(起始 2023-01-01)</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -3787,22 +3800,22 @@
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>expr=0 * * * *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 0 29 2 *;start=2023-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 * * * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 29 2 *', datetime.fromisoformat('2023-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 1, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 2, 29, 0, 0, tzinfo=datetime.timezone.utc)(2024 为闰年)</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 1, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 2, 29, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
@@ -3812,14 +3825,14 @@
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
-          <t>边界值(小时边界)</t>
+          <t>边界值(闰年边界)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-015</t>
+          <t>CRON-UT-017</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -3829,7 +3842,7 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>边界值:每月 1 号跨月(起始 01-02,月边界)</t>
+          <t>边界值:年末最后一分钟 23:59(起始 2024-01-01)</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -3854,22 +3867,22 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 1 * *;start=2024-01-02T00:00:00+00:00</t>
+          <t>expr=59 23 31 12 *;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 1 * *', datetime.fromisoformat('2024-01-02T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('59 23 31 12 *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 12, 31, 23, 59, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 12, 31, 23, 59, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L16" s="12" t="inlineStr">
@@ -3879,14 +3892,14 @@
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>边界值(月边界)</t>
+          <t>边界值(年边界 23:59)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="75" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-016</t>
+          <t>CRON-UT-018</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -3894,9 +3907,9 @@
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>边界值:闰年 2 月 29 日(起始 2023-01-01)</t>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>边界值:周日迭代(起始周六 01-06,星期边界)</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -3921,22 +3934,22 @@
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 29 2 *;start=2023-01-01T00:00:00+00:00</t>
+          <t>expr=0 0 * * 0;start=2024-01-06T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 29 2 *', datetime.fromisoformat('2023-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 * * 0', datetime.fromisoformat('2024-01-06T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 29, 0, 0, tzinfo=datetime.timezone.utc)(2024 为闰年)</t>
+          <t>datetime.datetime(2024, 1, 7, 0, 0, tzinfo=datetime.timezone.utc)(01-07 为周日)</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 29, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 7, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
@@ -3946,14 +3959,14 @@
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>边界值(闰年边界)</t>
+          <t>边界值(星期边界周日)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="75" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-017</t>
+          <t>CRON-UT-019</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -3961,9 +3974,9 @@
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>边界值:年末最后一分钟 23:59(起始 2024-01-01)</t>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>边界值:跨年 1 月 1 日(起始 2024-01-02,年边界)</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -3988,22 +4001,22 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>expr=59 23 31 12 *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 0 1 1 *;start=2024-01-02T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>croniter('59 23 31 12 *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 1 1 *', datetime.fromisoformat('2024-01-02T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 12, 31, 23, 59, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2025, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 12, 31, 23, 59, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2025, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L18" s="12" t="inlineStr">
@@ -4013,14 +4026,14 @@
       </c>
       <c r="M18" s="13" t="inlineStr">
         <is>
-          <t>边界值(年边界 23:59)</t>
+          <t>边界值(跨年边界)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-018</t>
+          <t>CRON-UT-020</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -4030,7 +4043,7 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>边界值:周日迭代(起始周六 01-06,星期边界)</t>
+          <t>边界值:步长 */15 非整点起步(起始 00:01)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -4055,22 +4068,22 @@
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 * * 0;start=2024-01-06T00:00:00+00:00</t>
+          <t>expr=*/15 * * * *;start=2024-01-01T00:01:00+00:00</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 * * 0', datetime.fromisoformat('2024-01-06T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('*/15 * * * *', datetime.fromisoformat('2024-01-01T00:01:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 7, 0, 0, tzinfo=datetime.timezone.utc)(01-07 为周日)</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 15, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 7, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 15, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -4080,14 +4093,14 @@
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
-          <t>边界值(星期边界周日)</t>
+          <t>边界值(步长边界)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="75" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-019</t>
+          <t>CRON-UT-021</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -4097,7 +4110,7 @@
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>边界值:跨年 1 月 1 日(起始 2024-01-02,年边界)</t>
+          <t>边界值:每月 1 号(起始 2024-01-01)</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -4122,22 +4135,22 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 1 1 *;start=2024-01-02T00:00:00+00:00</t>
+          <t>expr=0 0 1 * *;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 1 1 *', datetime.fromisoformat('2024-01-02T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 1 * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2025, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2025, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L20" s="12" t="inlineStr">
@@ -4147,14 +4160,14 @@
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>边界值(跨年边界)</t>
+          <t>边界值(月边界)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="75" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-020</t>
+          <t>CRON-UT-022</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -4164,7 +4177,7 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>边界值:步长 */15 非整点起步(起始 00:01)</t>
+          <t>边界值:周六迭代(起始周一 01-01,星期边界)</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -4182,29 +4195,29 @@
           <t>是</t>
         </is>
       </c>
-      <c r="G21" s="12" t="inlineStr">
+      <c r="G21" s="13" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>expr=*/15 * * * *;start=2024-01-01T00:01:00+00:00</t>
+          <t>expr=0 0 * * 6;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>croniter('*/15 * * * *', datetime.fromisoformat('2024-01-01T00:01:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 * * 6', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 15, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 6, 0, 0, tzinfo=datetime.timezone.utc)(01-06 为周六)</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 15, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 6, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
@@ -4214,14 +4227,14 @@
       </c>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>边界值(步长边界)</t>
+          <t>边界值(星期边界周六)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="75" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-021</t>
+          <t>CRON-UT-024</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -4229,9 +4242,9 @@
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>边界值:每月 1 号(起始 2024-01-01)</t>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>边界值:跨年(起始除夕 2023-12-31)</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -4256,22 +4269,22 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 1 * *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 0 1 1 *;start=2023-12-31T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 1 * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('0 0 1 1 *', datetime.fromisoformat('2023-12-31T00:00:00+00:00')).get_next(datetime)</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 2, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>datetime.datetime(2024, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
       <c r="L22" s="12" t="inlineStr">
@@ -4281,14 +4294,14 @@
       </c>
       <c r="M22" s="13" t="inlineStr">
         <is>
-          <t>边界值(月边界)</t>
+          <t>边界值(跨年边界)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="75" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-022</t>
+          <t>CRON-UT-042</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
@@ -4298,7 +4311,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>边界值:周六迭代(起始周一 01-01,星期边界)</t>
+          <t>边界值:6 段秒级表达式 */30 * * * * * 默认返回 float 时间戳</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -4316,29 +4329,29 @@
           <t>是</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 * * 6;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=*/30 * * * * *;start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>croniter('0 0 * * 6', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
+          <t>croniter('*/30 * * * * *', start).get_next()</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 6, 0, 0, tzinfo=datetime.timezone.utc)(01-06 为周六)</t>
+          <t>float(秒级时间戳,如 1704067201.0)</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>datetime.datetime(2024, 1, 6, 0, 0, tzinfo=datetime.timezone.utc)</t>
+          <t>float(秒级时间戳,如 1704067201.0)</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
@@ -4348,14 +4361,14 @@
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>边界值(星期边界周六)</t>
+          <t>边界值(秒级表达式,返回值类型)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="84" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-023</t>
+          <t>CRON-UT-043</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -4365,7 +4378,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>边界值:正午 12 点(起始 00:00)</t>
+          <t>边界值:夏令时切换日 0 2 * * *(America/New_York,2024-03-09 出发)</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -4390,485 +4403,284 @@
       </c>
       <c r="H24" s="12" t="inlineStr">
         <is>
-          <t>expr=0 12 * * *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 2 * * *;start=2024-03-09T00:00:00-05:00;tz=America/New_York</t>
         </is>
       </c>
       <c r="I24" s="12" t="inlineStr">
-        <is>
-          <t>croniter('0 12 * * *', datetime.fromisoformat('2024-01-01T00:00:00+00:00')).get_next(datetime)</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="inlineStr">
-        <is>
-          <t>datetime.datetime(2024, 1, 1, 12, 0, tzinfo=datetime.timezone.utc)</t>
-        </is>
-      </c>
-      <c r="K24" s="12" t="inlineStr">
-        <is>
-          <t>datetime.datetime(2024, 1, 1, 12, 0, tzinfo=datetime.timezone.utc)</t>
-        </is>
-      </c>
-      <c r="L24" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M24" s="13" t="inlineStr">
-        <is>
-          <t>边界值(正午边界)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="270" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-024</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>get_next()/get_prev() 迭代</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>边界值:跨年(起始除夕 2023-12-31)</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G25" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
-        <is>
-          <t>expr=0 0 1 1 *;start=2023-12-31T00:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="I25" s="12" t="inlineStr">
-        <is>
-          <t>croniter('0 0 1 1 *', datetime.fromisoformat('2023-12-31T00:00:00+00:00')).get_next(datetime)</t>
-        </is>
-      </c>
-      <c r="J25" s="12" t="inlineStr">
-        <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
-        </is>
-      </c>
-      <c r="K25" s="12" t="inlineStr">
-        <is>
-          <t>datetime.datetime(2024, 1, 1, 0, 0, tzinfo=datetime.timezone.utc)</t>
-        </is>
-      </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M25" s="13" t="inlineStr">
-        <is>
-          <t>边界值(跨年边界)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="270" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-042</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>get_next()/get_prev() 迭代</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>边界值:6 段秒级表达式 */30 * * * * * 默认返回 float 时间戳</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H26" s="12" t="inlineStr">
-        <is>
-          <t>expr=*/30 * * * * *;start=2024-01-01T00:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="I26" s="12" t="inlineStr">
-        <is>
-          <t>croniter('*/30 * * * * *', start).get_next()</t>
-        </is>
-      </c>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>float(秒级时间戳,如 1704067201.0)</t>
-        </is>
-      </c>
-      <c r="K26" s="12" t="inlineStr">
-        <is>
-          <t>float(秒级时间戳,如 1704067201.0)</t>
-        </is>
-      </c>
-      <c r="L26" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M26" s="13" t="inlineStr">
-        <is>
-          <t>边界值(秒级表达式,返回值类型)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="270" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-043</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>get_next()/get_prev() 迭代</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>边界值:夏令时切换日 0 2 * * *(America/New_York,2024-03-09 出发)</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H27" s="12" t="inlineStr">
-        <is>
-          <t>expr=0 2 * * *;start=2024-03-09T00:00:00-05:00;tz=America/New_York</t>
-        </is>
-      </c>
-      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>from zoneinfo import ZoneInfo
 start = datetime.fromisoformat('2024-03-09T00:00:00-05:00').replace(tzinfo=ZoneInfo('America/New_York'))
 croniter('0 2 * * *', start).get_next(datetime)</t>
         </is>
       </c>
-      <c r="J27" s="12" t="inlineStr">
+      <c r="J24" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 3, 9, 2, 0, tzinfo=ZoneInfo('America/New_York'))(切换日前一天,02:00 仍存在)</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr">
+      <c r="K24" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 3, 9, 2, 0, tzinfo=ZoneInfo('America/New_York'))(切换日前一天,02:00 仍存在)</t>
         </is>
       </c>
-      <c r="L27" s="12" t="inlineStr">
+      <c r="L24" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M27" s="13" t="inlineStr">
+      <c r="M24" s="13" t="inlineStr">
         <is>
           <t>边界值(夏令时/ZoneInfo 时区)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="270" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="25" ht="270" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-044</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>边界值:非法起始时间类型(object)应抛 TypeError/ValueError</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G28" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H28" s="12" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>expr=* * * * *;start=object()</t>
         </is>
       </c>
-      <c r="I28" s="12" t="inlineStr">
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>croniter('* * * * *', object()).get_next()</t>
         </is>
       </c>
-      <c r="J28" s="12" t="inlineStr">
+      <c r="J25" s="12" t="inlineStr">
         <is>
           <t>TypeError 或 ValueError</t>
         </is>
       </c>
-      <c r="K28" s="12" t="inlineStr">
+      <c r="K25" s="12" t="inlineStr">
         <is>
           <t>TypeError 或 ValueError</t>
         </is>
       </c>
-      <c r="L28" s="12" t="inlineStr">
+      <c r="L25" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M28" s="13" t="inlineStr">
+      <c r="M25" s="13" t="inlineStr">
         <is>
           <t>异常测试(非法输入类型)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="270" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="26" ht="270" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-051</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>边界值:春季夏令时跳变日 0 2 * * *(2024-03-10,America/New_York)</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H29" s="12" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
         <is>
           <t>expr=0 2 * * *;start=2024-03-10T00:00:00-05:00;tz=America/New_York</t>
         </is>
       </c>
-      <c r="I29" s="12" t="inlineStr">
+      <c r="I26" s="12" t="inlineStr">
         <is>
           <t>from zoneinfo import ZoneInfo
 start = datetime.fromisoformat('2024-03-10T00:00:00-05:00').replace(tzinfo=ZoneInfo('America/New_York'))
 croniter('0 2 * * *', start).get_next(datetime)</t>
         </is>
       </c>
-      <c r="J29" s="12" t="inlineStr">
+      <c r="J26" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 3, 10, 3, 0, tzinfo=ZoneInfo('America/New_York'))(02:00 因夏令时开始不存在,自动顺延到 03:00 EDT)</t>
         </is>
       </c>
-      <c r="K29" s="12" t="inlineStr">
+      <c r="K26" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 3, 10, 3, 0, tzinfo=ZoneInfo('America/New_York'))(02:00 因夏令时开始不存在,自动顺延到 03:00 EDT)</t>
         </is>
       </c>
-      <c r="L29" s="12" t="inlineStr">
+      <c r="L26" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M29" s="13" t="inlineStr">
+      <c r="M26" s="13" t="inlineStr">
         <is>
           <t>边界值(夏令时跳变,不存在的本地时刻)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="270" customHeight="1">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="27" ht="270" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-052</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>边界值:秋季夏令时回拨日 0 1 * * *(2024-11-03,America/New_York)</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>expr=0 1 * * *;start=2024-11-03T00:00:00-04:00;tz=America/New_York</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>from zoneinfo import ZoneInfo
 start = datetime.fromisoformat('2024-11-03T00:00:00-04:00').replace(tzinfo=ZoneInfo('America/New_York'))
 croniter('0 1 * * *', start).get_next(datetime)</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 11, 3, 1, 0, tzinfo=ZoneInfo('America/New_York'))(01:00 在回拨日出现两次,取第一次 EDT,UTC 05:00)</t>
         </is>
       </c>
-      <c r="K30" s="12" t="inlineStr">
+      <c r="K27" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 11, 3, 1, 0, tzinfo=ZoneInfo('America/New_York'))(01:00 在回拨日出现两次,取第一次 EDT,UTC 05:00)</t>
         </is>
       </c>
-      <c r="L30" s="12" t="inlineStr">
+      <c r="L27" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M30" s="13" t="inlineStr">
+      <c r="M27" s="13" t="inlineStr">
         <is>
           <t>边界值(夏令时回拨,歧义本地时刻取第一次)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="194" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="28" ht="270" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-025</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>连续迭代场景:get_next()/get_prev()</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>场景:连续两次迭代间隔恰为 10 分钟且 get_prev 早于起点</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H31" s="12" t="inlineStr">
+      <c r="H28" s="12" t="inlineStr">
         <is>
           <t>expr=*/10 * * * *;start=2024-01-15T12:00:00+00:00</t>
         </is>
       </c>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="I28" s="12" t="inlineStr">
         <is>
           <t>s = datetime.fromisoformat('2024-01-15T12:00:00+00:00')
 it = croniter('*/10 * * * *', s)
@@ -4877,71 +4689,71 @@
 croniter('*/10 * * * *', s).get_prev(datetime)</t>
         </is>
       </c>
-      <c r="J31" s="12" t="inlineStr">
+      <c r="J28" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 10, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 20, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))
 datetime.datetime(2024, 1, 15, 11, 50, fold=1, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
-      <c r="K31" s="12" t="inlineStr">
+      <c r="K28" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 10, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 20, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))
 datetime.datetime(2024, 1, 15, 11, 50, fold=1, tzinfo=datetime.timezone.utc)</t>
         </is>
       </c>
-      <c r="L31" s="12" t="inlineStr">
+      <c r="L28" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M31" s="13" t="inlineStr">
+      <c r="M28" s="13" t="inlineStr">
         <is>
           <t>场景法(连续迭代状态)</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="278" customHeight="1">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="29" ht="270" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-033</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>croniter() 解析</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>零步长范围 0 0 * * 5-5/0 应抛出标准 CroniterBadCronError</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H32" s="12" t="inlineStr">
+      <c r="H29" s="12" t="inlineStr">
         <is>
           <t>expr=0 0 * * 5-5/0(零步长范围);start=2024-01-01T00:00:00+00:00</t>
         </is>
       </c>
-      <c r="I32" s="12" t="inlineStr">
+      <c r="I29" s="12" t="inlineStr">
         <is>
           <t>try:
     croniter('0 0 * * 5-5/0', datetime.fromisoformat('2024-01-01T00:00:00+00:00'))
@@ -4952,205 +4764,205 @@
     print('ValueError:', e)</t>
         </is>
       </c>
-      <c r="J32" s="12" t="inlineStr">
+      <c r="J29" s="12" t="inlineStr">
         <is>
           <t>CroniterBadCronError: [0 0 * * 5-5/0] step must be greater than zero</t>
         </is>
       </c>
-      <c r="K32" s="12" t="inlineStr">
+      <c r="K29" s="12" t="inlineStr">
         <is>
           <t>ValueError: range() arg 3 must not be zero</t>
         </is>
       </c>
-      <c r="L32" s="12" t="inlineStr">
+      <c r="L29" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="M32" s="13" t="inlineStr">
+      <c r="M29" s="13" t="inlineStr">
         <is>
           <t>等价类(非法表达式类,星期字段零步长)；基线 6.2.2 抛裸 ValueError:range() arg 3 must not be zero,不属于 CroniterError 家族</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="210" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="30" ht="270" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-034</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>边界值:expand_from_start_time 月份步进低界 0 0 1 */2 *(CRON-D-002,issue #235)</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H33" s="12" t="inlineStr">
+      <c r="H30" s="12" t="inlineStr">
         <is>
           <t>expr=0 0 1 */2 *;start=2024-02-01T00:00:00+00:00;expand_from_start_time=True</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I30" s="12" t="inlineStr">
         <is>
           <t>it = croniter('0 0 1 */2 *', datetime.fromisoformat('2024-02-01T00:00:00+00:00'), expand_from_start_time=True)
 it.get_next(datetime)</t>
         </is>
       </c>
-      <c r="J33" s="12" t="inlineStr">
+      <c r="J30" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 4, 1, 0, 0, tzinfo=datetime.timezone.utc)(expand 下首次触发;完整序列 2024-04-01、06-01、08-01、10-01)</t>
         </is>
       </c>
-      <c r="K33" s="12" t="inlineStr">
+      <c r="K30" s="12" t="inlineStr">
         <is>
           <t>CroniterBadCronError: [0 0 1 */2 *] is not acceptable, out of range</t>
         </is>
       </c>
-      <c r="L33" s="12" t="inlineStr">
+      <c r="L30" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="M33" s="13" t="inlineStr">
+      <c r="M30" s="13" t="inlineStr">
         <is>
           <t>边界值(月份步进低界,expand_from_start_time=True)基线 6.2.2 从 2024-02-01 出发直接报 CroniterBadCronError out of range(月份低界余数为 0 时得到非法月份 0);修复后正常返回 04-01 起</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="225" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
+    <row r="31" ht="194" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-035</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>get_next()/get_prev() 迭代</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>边界值:Sunday 步进低界 0 0 * * 1-7/2(CRON-D-003,issue #239)</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G34" s="12" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H34" s="12" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
         <is>
           <t>expr=0 0 * * 1-7/2;start=2024-01-07T00:00:00+00:00(周日);expand_from_start_time=True</t>
         </is>
       </c>
-      <c r="I34" s="12" t="inlineStr">
+      <c r="I31" s="12" t="inlineStr">
         <is>
           <t>it = croniter('0 0 * * 1-7/2', datetime.fromisoformat('2024-01-07T00:00:00+00:00'), expand_from_start_time=True)
 it.get_next(datetime)</t>
         </is>
       </c>
-      <c r="J34" s="12" t="inlineStr">
+      <c r="J31" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 1, 9, 0, 0, tzinfo=datetime.timezone.utc)(expand 下首次触发;完整序列 01-09、01-11、01-13、01-14)</t>
         </is>
       </c>
-      <c r="K34" s="12" t="inlineStr">
+      <c r="K31" s="12" t="inlineStr">
         <is>
           <t>datetime.datetime(2024, 1, 8, 0, 0, tzinfo=datetime.timezone.utc)(expand 下首次触发;完整序列 01-08、01-10、01-12、01-14)</t>
         </is>
       </c>
-      <c r="L34" s="12" t="inlineStr">
+      <c r="L31" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="M34" s="13" t="inlineStr">
+      <c r="M31" s="13" t="inlineStr">
         <is>
           <t>边界值(周日步进低界,expand_from_start_time=True)基线 6.2.2 从周日出发返回 01-08、01-10、01-12(相位错位一天,weekday()+1 将 Sunday 映射为 7 而非 0);修复后返回 01-09 起</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="210" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="32" ht="278" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-037</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>连续迭代场景:get_next()/get_prev()</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>场景:步长范围 5-59/10 连续两次结果恰为 10 分钟且 get_prev 有效</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H35" s="12" t="inlineStr">
+      <c r="H32" s="12" t="inlineStr">
         <is>
           <t>expr=5-59/10 * * * *;start=2024-01-15T12:00:00+00:00</t>
         </is>
       </c>
-      <c r="I35" s="12" t="inlineStr">
+      <c r="I32" s="12" t="inlineStr">
         <is>
           <t>s = datetime.fromisoformat('2024-01-15T12:00:00+00:00')
 it = croniter('5-59/10 * * * *', s)
@@ -5159,69 +4971,69 @@
 croniter('5-59/10 * * * *', s).get_prev(datetime)</t>
         </is>
       </c>
-      <c r="J35" s="12" t="inlineStr">
+      <c r="J32" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 5, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 15, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="K35" s="12" t="inlineStr">
+      <c r="K32" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 5, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 15, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="L35" s="12" t="inlineStr">
+      <c r="L32" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M35" s="13" t="inlineStr">
+      <c r="M32" s="13" t="inlineStr">
         <is>
           <t>场景法(步长范围)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="270" customHeight="1">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="33" ht="210" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-038</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>连续迭代场景:get_next()/get_prev()</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>场景:枚举列表 0,10,20,30,40,50 连续两次结果恰为 10 分钟且 get_prev 有效</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G36" s="12" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H36" s="12" t="inlineStr">
+      <c r="H33" s="12" t="inlineStr">
         <is>
           <t>expr=0,10,20,30,40,50 * * * *;start=2024-01-15T12:00:00+00:00</t>
         </is>
       </c>
-      <c r="I36" s="12" t="inlineStr">
+      <c r="I33" s="12" t="inlineStr">
         <is>
           <t>s = datetime.fromisoformat('2024-01-15T12:00:00+00:00')
 it = croniter('0,10,20,30,40,50 * * * *', s)
@@ -5230,69 +5042,69 @@
 croniter('0,10,20,30,40,50 * * * *', s).get_prev(datetime)</t>
         </is>
       </c>
-      <c r="J36" s="12" t="inlineStr">
+      <c r="J33" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 10, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 20, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="K36" s="12" t="inlineStr">
+      <c r="K33" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 1, 15, 12, 10, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 1, 15, 12, 20, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="L36" s="12" t="inlineStr">
+      <c r="L33" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M36" s="13" t="inlineStr">
+      <c r="M33" s="13" t="inlineStr">
         <is>
           <t>场景法(枚举列表)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="67.5" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="34" ht="225" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-039</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>连续迭代场景:get_next()/get_prev()</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>场景:跨日跨月 */10 从 06-30T23:50 出发连续两次结果恰为 10 分钟且 get_prev 有效</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G37" s="12" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H37" s="12" t="inlineStr">
+      <c r="H34" s="12" t="inlineStr">
         <is>
           <t>expr=*/10 * * * *;start=2024-06-30T23:50:00+00:00</t>
         </is>
       </c>
-      <c r="I37" s="12" t="inlineStr">
+      <c r="I34" s="12" t="inlineStr">
         <is>
           <t>s = datetime.fromisoformat('2024-06-30T23:50:00+00:00')
 it = croniter('*/10 * * * *', s)
@@ -5301,70 +5113,70 @@
 croniter('*/10 * * * *', s).get_prev(datetime)</t>
         </is>
       </c>
-      <c r="J37" s="12" t="inlineStr">
+      <c r="J34" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 7, 1, 0, 0, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 7, 1, 0, 10, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="K37" s="12" t="inlineStr">
+      <c r="K34" s="12" t="inlineStr">
         <is>
           <t>(datetime.datetime(2024, 7, 1, 0, 0, tzinfo=datetime.timezone.utc), datetime.datetime(2024, 7, 1, 0, 10, tzinfo=datetime.timezone.utc), datetime.timedelta(seconds=600))</t>
         </is>
       </c>
-      <c r="L37" s="12" t="inlineStr">
+      <c r="L34" s="12" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="M37" s="13" t="inlineStr">
+      <c r="M34" s="13" t="inlineStr">
         <is>
           <t>场景法(跨日跨月)</t>
         </is>
       </c>
-      <c r="O37" s="1" t="n"/>
-    </row>
-    <row r="38" ht="67.5" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="O34" s="1" t="n"/>
+    </row>
+    <row r="35" ht="210" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>CRON-UT-040</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>连续迭代场景:get_next()/get_prev()</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>场景:时区偏移 +09:00 */10 连续两次结果恰为 10 分钟且 get_prev 有效</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
         <is>
           <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
         </is>
       </c>
-      <c r="H38" s="12" t="inlineStr">
+      <c r="H35" s="12" t="inlineStr">
         <is>
           <t>expr=*/10 * * * *;start=2024-08-01T00:05:00+09:00</t>
         </is>
       </c>
-      <c r="I38" s="12" t="inlineStr">
+      <c r="I35" s="12" t="inlineStr">
         <is>
           <t>s = datetime.fromisoformat('2024-08-01T00:05:00+09:00')
 it = croniter('*/10 * * * *', s)
@@ -5373,14 +5185,217 @@
 croniter('*/10 * * * *', s).get_prev(datetime)</t>
         </is>
       </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>(datetime.datetime(2024, 8, 1, 0, 10, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.datetime(2024, 8, 1, 0, 20, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.timedelta(seconds=600))</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>(datetime.datetime(2024, 8, 1, 0, 10, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.datetime(2024, 8, 1, 0, 20, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.timedelta(seconds=600))</t>
+        </is>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M35" s="13" t="inlineStr">
+        <is>
+          <t>场景法(时区偏移)</t>
+        </is>
+      </c>
+      <c r="O35" s="1" t="n"/>
+    </row>
+    <row r="36" ht="270" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>CRON-UT-045</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>match:整点时刻 0 0 * * * 在 00:00 命中</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>expr=0 0 * * *;start=2024-01-01T00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>croniter.match('0 0 * * *', start)</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>True(该时刻符合规则)</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>True(该时刻符合规则)</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M36" s="13" t="inlineStr">
+        <is>
+          <t>等价类(时刻命中类)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="67.5" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>CRON-UT-046</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>match:整点时刻 0 0 * * * 在 00:01 未命中</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>expr=0 0 * * *;start=2024-01-01T00:01:00+00:00</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>croniter.match('0 0 * * *', start)</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>False(该时刻不符合规则)</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>False(该时刻不符合规则)</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M37" s="13" t="inlineStr">
+        <is>
+          <t>等价类(时刻未命中类)</t>
+        </is>
+      </c>
+      <c r="O37" s="1" t="n"/>
+    </row>
+    <row r="38" ht="67.5" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>CRON-UT-047</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>match_range:一天窗口内存在整点触发点</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>expr=0 0 * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-02T00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>croniter.match_range('0 0 * * *', start, end)</t>
+        </is>
+      </c>
       <c r="J38" s="12" t="inlineStr">
         <is>
-          <t>(datetime.datetime(2024, 8, 1, 0, 10, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.datetime(2024, 8, 1, 0, 20, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.timedelta(seconds=600))</t>
+          <t>True(窗口内存在触发点)</t>
         </is>
       </c>
       <c r="K38" s="12" t="inlineStr">
         <is>
-          <t>(datetime.datetime(2024, 8, 1, 0, 10, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.datetime(2024, 8, 1, 0, 20, tzinfo=datetime.timezone(datetime.timedelta(seconds=32400))), datetime.timedelta(seconds=600))</t>
+          <t>True(窗口内存在触发点)</t>
         </is>
       </c>
       <c r="L38" s="12" t="inlineStr">
@@ -5390,15 +5405,14 @@
       </c>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>场景法(时区偏移)</t>
-        </is>
-      </c>
-      <c r="O38" s="1" t="n"/>
+          <t>等价类(窗口含触发点类)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="75" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-045</t>
+          <t>CRON-UT-048</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
@@ -5408,7 +5422,7 @@
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>match:整点时刻 0 0 * * * 在 00:00 命中</t>
+          <t>match_range:半小时窗口内不存在 01:00 触发点</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -5433,22 +5447,22 @@
       </c>
       <c r="H39" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 * * *;start=2024-01-01T00:00:00+00:00</t>
+          <t>expr=0 1 * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-01T00:30:00+00:00</t>
         </is>
       </c>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>croniter.match('0 0 * * *', start)</t>
+          <t>croniter.match_range('0 1 * * *', start, end)</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
         <is>
-          <t>True(该时刻符合规则)</t>
+          <t>False(窗口内不存在触发点)</t>
         </is>
       </c>
       <c r="K39" s="12" t="inlineStr">
         <is>
-          <t>True(该时刻符合规则)</t>
+          <t>False(窗口内不存在触发点)</t>
         </is>
       </c>
       <c r="L39" s="12" t="inlineStr">
@@ -5458,14 +5472,14 @@
       </c>
       <c r="M39" s="13" t="inlineStr">
         <is>
-          <t>等价类(时刻命中类)</t>
+          <t>等价类(窗口不含触发点类)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="75" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-046</t>
+          <t>CRON-UT-049</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
@@ -5475,7 +5489,7 @@
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>match:整点时刻 0 0 * * * 在 00:01 未命中</t>
+          <t>is_valid:6 段秒级表达式 0 0 0 1 1 *(second_at_beginning=True)合法</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -5500,22 +5514,22 @@
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 * * *;start=2024-01-01T00:01:00+00:00</t>
+          <t>expr=0 0 0 1 1 *;second_at_beginning=True</t>
         </is>
       </c>
       <c r="I40" s="12" t="inlineStr">
         <is>
-          <t>croniter.match('0 0 * * *', start)</t>
+          <t>croniter.is_valid('0 0 0 1 1 *', second_at_beginning=True)</t>
         </is>
       </c>
       <c r="J40" s="12" t="inlineStr">
         <is>
-          <t>False(该时刻不符合规则)</t>
+          <t>True(表达式合法)</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
         <is>
-          <t>False(该时刻不符合规则)</t>
+          <t>True(表达式合法)</t>
         </is>
       </c>
       <c r="L40" s="12" t="inlineStr">
@@ -5525,15 +5539,14 @@
       </c>
       <c r="M40" s="13" t="inlineStr">
         <is>
-          <t>等价类(时刻未命中类)</t>
-        </is>
-      </c>
-      <c r="O40" s="1" t="n"/>
+          <t>等价类(合法表达式类,秒级)</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="67.5" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>CRON-UT-047</t>
+          <t>CRON-UT-050</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
@@ -5543,7 +5556,7 @@
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>match_range:一天窗口内存在整点触发点</t>
+          <t>croniter_range:3 分钟窗口内触发点个数为 4</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
@@ -5568,22 +5581,22 @@
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>expr=0 0 * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-02T00:00:00+00:00</t>
+          <t>expr=* * * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-01T00:03:00+00:00</t>
         </is>
       </c>
       <c r="I41" s="12" t="inlineStr">
         <is>
-          <t>croniter.match_range('0 0 * * *', start, end)</t>
+          <t>list(croniter_range(start, end, '* * * * *'))</t>
         </is>
       </c>
       <c r="J41" s="12" t="inlineStr">
         <is>
-          <t>True(窗口内存在触发点)</t>
+          <t>len == 4(00:00、00:01、00:02、00:03)</t>
         </is>
       </c>
       <c r="K41" s="12" t="inlineStr">
         <is>
-          <t>True(窗口内存在触发点)</t>
+          <t>len == 4(00:00、00:01、00:02、00:03)</t>
         </is>
       </c>
       <c r="L41" s="12" t="inlineStr">
@@ -5593,210 +5606,54 @@
       </c>
       <c r="M41" s="13" t="inlineStr">
         <is>
-          <t>等价类(窗口含触发点类)</t>
+          <t>场景法(窗口内连续触发序列)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="75" customHeight="1">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-048</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>match_range:半小时窗口内不存在 01:00 触发点</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G42" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H42" s="12" t="inlineStr">
-        <is>
-          <t>expr=0 1 * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-01T00:30:00+00:00</t>
-        </is>
-      </c>
-      <c r="I42" s="12" t="inlineStr">
-        <is>
-          <t>croniter.match_range('0 1 * * *', start, end)</t>
-        </is>
-      </c>
-      <c r="J42" s="12" t="inlineStr">
-        <is>
-          <t>False(窗口内不存在触发点)</t>
-        </is>
-      </c>
-      <c r="K42" s="12" t="inlineStr">
-        <is>
-          <t>False(窗口内不存在触发点)</t>
-        </is>
-      </c>
-      <c r="L42" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M42" s="13" t="inlineStr">
-        <is>
-          <t>等价类(窗口不含触发点类)</t>
-        </is>
-      </c>
+      <c r="A42" s="12" t="n"/>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12" t="n"/>
+      <c r="M42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-049</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>is_valid:6 段秒级表达式 0 0 0 1 1 *(second_at_beginning=True)合法</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G43" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H43" s="12" t="inlineStr">
-        <is>
-          <t>expr=0 0 0 1 1 *;second_at_beginning=True</t>
-        </is>
-      </c>
-      <c r="I43" s="12" t="inlineStr">
-        <is>
-          <t>croniter.is_valid('0 0 0 1 1 *', second_at_beginning=True)</t>
-        </is>
-      </c>
-      <c r="J43" s="12" t="inlineStr">
-        <is>
-          <t>True(表达式合法)</t>
-        </is>
-      </c>
-      <c r="K43" s="12" t="inlineStr">
-        <is>
-          <t>True(表达式合法)</t>
-        </is>
-      </c>
-      <c r="L43" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M43" s="13" t="inlineStr">
-        <is>
-          <t>等价类(合法表达式类,秒级)</t>
-        </is>
-      </c>
+      <c r="A43" s="12" t="n"/>
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="12" t="n"/>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="12" t="n"/>
+      <c r="K43" s="12" t="n"/>
+      <c r="L43" s="12" t="n"/>
+      <c r="M43" s="12" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
-        <is>
-          <t>CRON-UT-050</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>匹配与范围校验:match/match_range/croniter_range/is_valid</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>croniter_range:3 分钟窗口内触发点个数为 4</t>
-        </is>
-      </c>
-      <c r="D44" s="12" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G44" s="12" t="inlineStr">
-        <is>
-          <t>安装 croniter 6.2.2；准备固定输入和基准时间</t>
-        </is>
-      </c>
-      <c r="H44" s="12" t="inlineStr">
-        <is>
-          <t>expr=* * * * *;start=2024-01-01T00:00:00+00:00;end=2024-01-01T00:03:00+00:00</t>
-        </is>
-      </c>
-      <c r="I44" s="12" t="inlineStr">
-        <is>
-          <t>list(croniter_range(start, end, '* * * * *'))</t>
-        </is>
-      </c>
-      <c r="J44" s="12" t="inlineStr">
-        <is>
-          <t>len == 4(00:00、00:01、00:02、00:03)</t>
-        </is>
-      </c>
-      <c r="K44" s="12" t="inlineStr">
-        <is>
-          <t>len == 4(00:00、00:01、00:02、00:03)</t>
-        </is>
-      </c>
-      <c r="L44" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="M44" s="13" t="inlineStr">
-        <is>
-          <t>场景法(窗口内连续触发序列)</t>
-        </is>
-      </c>
+      <c r="A44" s="12" t="n"/>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
+      <c r="H44" s="12" t="n"/>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
+      <c r="K44" s="12" t="n"/>
+      <c r="L44" s="12" t="n"/>
+      <c r="M44" s="12" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="12" t="n"/>
@@ -5823,55 +5680,10 @@
       <c r="G46" s="12" t="n"/>
       <c r="H46" s="12" t="n"/>
       <c r="I46" s="12" t="n"/>
-      <c r="J46" s="12" t="n"/>
+      <c r="J46" s="13" t="n"/>
       <c r="K46" s="12" t="n"/>
       <c r="L46" s="12" t="n"/>
       <c r="M46" s="12" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="n"/>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="12" t="n"/>
-      <c r="I47" s="12" t="n"/>
-      <c r="J47" s="12" t="n"/>
-      <c r="K47" s="12" t="n"/>
-      <c r="L47" s="12" t="n"/>
-      <c r="M47" s="12" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="12" t="n"/>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="n"/>
-      <c r="E48" s="12" t="n"/>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="12" t="n"/>
-      <c r="I48" s="12" t="n"/>
-      <c r="J48" s="12" t="n"/>
-      <c r="K48" s="12" t="n"/>
-      <c r="L48" s="12" t="n"/>
-      <c r="M48" s="12" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="n"/>
-      <c r="B49" s="12" t="n"/>
-      <c r="C49" s="12" t="n"/>
-      <c r="D49" s="12" t="n"/>
-      <c r="E49" s="12" t="n"/>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="12" t="n"/>
-      <c r="H49" s="12" t="n"/>
-      <c r="I49" s="12" t="n"/>
-      <c r="J49" s="13" t="n"/>
-      <c r="K49" s="12" t="n"/>
-      <c r="L49" s="12" t="n"/>
-      <c r="M49" s="12" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>